<commit_message>
se realizaron los cálculos correspondientes a la deflexion teorica
</commit_message>
<xml_diff>
--- a/Analysis/Cálculos.xlsx
+++ b/Analysis/Cálculos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\david\Documents\Evaluacion 1 Herramientas\Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66AB6E54-3D90-4E98-BA4B-B77809E76C93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8678DB06-72F3-411F-A14D-A36F3E49729D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="23">
   <si>
     <t>Carga [KN]</t>
   </si>
@@ -81,12 +81,39 @@
   </si>
   <si>
     <t xml:space="preserve">Transformación de unidades </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calculo de defleccion teorica de Euler-Bernoulli </t>
+  </si>
+  <si>
+    <t>Carga (P) [N]</t>
+  </si>
+  <si>
+    <t>Delta_teo [m]</t>
+  </si>
+  <si>
+    <t>Segundo momento de área</t>
+  </si>
+  <si>
+    <t>[m^4]</t>
+  </si>
+  <si>
+    <t>Cálculo segundo momento de área</t>
+  </si>
+  <si>
+    <t>I = (b*(h)^3)/12</t>
+  </si>
+  <si>
+    <t>Delta_teo = (P*(L^3))/(48*E*I)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="201" formatCode="0.00000"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -104,7 +131,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -123,8 +150,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -147,11 +186,37 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -163,19 +228,40 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="201" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="201" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -456,41 +542,41 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:J44"/>
+  <dimension ref="B2:J52"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="9.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.44140625" customWidth="1"/>
-    <col min="5" max="5" width="29.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.33203125" customWidth="1"/>
+    <col min="3" max="3" width="23.21875" customWidth="1"/>
+    <col min="5" max="5" width="30" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="1"/>
-      <c r="E4" s="1" t="s">
+      <c r="C4" s="8"/>
+      <c r="E4" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
+      <c r="F4" s="8"/>
+      <c r="G4" s="8"/>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="1" t="s">
         <v>1</v>
       </c>
       <c r="E5" s="2" t="s">
@@ -622,13 +708,13 @@
       </c>
       <c r="F18" s="7"/>
       <c r="G18" s="7"/>
-      <c r="J18" s="9"/>
+      <c r="J18" s="6"/>
     </row>
     <row r="19" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B19" s="8" t="s">
+      <c r="B19" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C19" s="8" t="s">
+      <c r="C19" s="5" t="s">
         <v>11</v>
       </c>
       <c r="E19" s="2" t="s">
@@ -643,11 +729,11 @@
     </row>
     <row r="20" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B20" s="3">
-        <f>B6*1000</f>
+        <f t="shared" ref="B20:B28" si="0">B6*1000</f>
         <v>0</v>
       </c>
       <c r="C20" s="3">
-        <f>C6/1000</f>
+        <f t="shared" ref="C20:C28" si="1">C6/1000</f>
         <v>0</v>
       </c>
       <c r="E20" s="2" t="s">
@@ -662,11 +748,11 @@
     </row>
     <row r="21" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B21" s="3">
-        <f>B7*1000</f>
+        <f t="shared" si="0"/>
         <v>5000</v>
       </c>
-      <c r="C21" s="3">
-        <f>C7/1000</f>
+      <c r="C21" s="16">
+        <f t="shared" si="1"/>
         <v>2.6000000000000003E-4</v>
       </c>
       <c r="E21" s="2" t="s">
@@ -681,11 +767,11 @@
     </row>
     <row r="22" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B22" s="3">
-        <f>B8*1000</f>
+        <f t="shared" si="0"/>
         <v>10000</v>
       </c>
       <c r="C22" s="3">
-        <f>C8/1000</f>
+        <f t="shared" si="1"/>
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="E22" s="2" t="s">
@@ -701,69 +787,257 @@
     </row>
     <row r="23" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B23" s="3">
-        <f>B9*1000</f>
+        <f t="shared" si="0"/>
         <v>15000</v>
       </c>
       <c r="C23" s="3">
-        <f>C9/1000</f>
+        <f t="shared" si="1"/>
         <v>7.6000000000000004E-4</v>
       </c>
     </row>
     <row r="24" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B24" s="3">
-        <f>B10*1000</f>
+        <f t="shared" si="0"/>
         <v>20000</v>
       </c>
       <c r="C24" s="3">
-        <f>C10/1000</f>
+        <f t="shared" si="1"/>
         <v>1.01E-3</v>
       </c>
     </row>
     <row r="25" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B25" s="3">
-        <f>B11*1000</f>
+        <f t="shared" si="0"/>
         <v>25000</v>
       </c>
       <c r="C25" s="3">
-        <f>C11/1000</f>
+        <f t="shared" si="1"/>
         <v>1.2800000000000001E-3</v>
       </c>
     </row>
     <row r="26" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B26" s="3">
-        <f>B12*1000</f>
+        <f t="shared" si="0"/>
         <v>30000</v>
       </c>
       <c r="C26" s="3">
-        <f>C12/1000</f>
+        <f t="shared" si="1"/>
         <v>1.5400000000000001E-3</v>
       </c>
     </row>
     <row r="27" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B27" s="3">
-        <f>B13*1000</f>
+        <f t="shared" si="0"/>
         <v>35000</v>
       </c>
       <c r="C27" s="3">
-        <f>C13/1000</f>
+        <f t="shared" si="1"/>
         <v>1.7700000000000001E-3</v>
       </c>
     </row>
     <row r="28" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B28" s="3">
-        <f>B14*1000</f>
+        <f t="shared" si="0"/>
         <v>40000</v>
       </c>
       <c r="C28" s="3">
-        <f>C14/1000</f>
+        <f t="shared" si="1"/>
         <v>2.0499999999999997E-3</v>
       </c>
     </row>
-    <row r="44" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E44" s="9"/>
+    <row r="31" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B31" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="C31" s="10"/>
+      <c r="D31" s="10"/>
+      <c r="E31" s="10"/>
+    </row>
+    <row r="32" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B32" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C32" s="10"/>
+      <c r="D32" s="10"/>
+      <c r="E32" s="10"/>
+    </row>
+    <row r="33" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B33" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="C33" s="13"/>
+      <c r="D33" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E33" s="4">
+        <f>(G20*(G21)^3)/12</f>
+        <v>1.0666666666666669E-3</v>
+      </c>
+    </row>
+    <row r="39" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B39" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="C39" s="14"/>
+      <c r="D39" s="14"/>
+      <c r="E39" s="14"/>
+    </row>
+    <row r="40" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B40" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="C40" s="14"/>
+      <c r="D40" s="14"/>
+      <c r="E40" s="14"/>
+    </row>
+    <row r="41" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B41" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="C41" s="11"/>
+      <c r="D41" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="E41" s="11"/>
+    </row>
+    <row r="42" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B42" s="11">
+        <f>B20</f>
+        <v>0</v>
+      </c>
+      <c r="C42" s="11"/>
+      <c r="D42" s="11">
+        <f>B42*(($G$19)^3)/48*$E$33*$G$22</f>
+        <v>0</v>
+      </c>
+      <c r="E42" s="11"/>
+    </row>
+    <row r="43" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B43" s="11">
+        <f>B21</f>
+        <v>5000</v>
+      </c>
+      <c r="C43" s="11"/>
+      <c r="D43" s="15">
+        <f>B43*(($G$19)^3)/(48*$E$33*$G$22)</f>
+        <v>2.4999999999999995E-4</v>
+      </c>
+      <c r="E43" s="15"/>
+    </row>
+    <row r="44" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B44" s="11">
+        <f>B22</f>
+        <v>10000</v>
+      </c>
+      <c r="C44" s="11"/>
+      <c r="D44" s="15">
+        <f t="shared" ref="D44:D50" si="2">B44*(($G$19)^3)/(48*$E$33*$G$22)</f>
+        <v>4.999999999999999E-4</v>
+      </c>
+      <c r="E44" s="15"/>
+    </row>
+    <row r="45" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B45" s="11">
+        <f>B23</f>
+        <v>15000</v>
+      </c>
+      <c r="C45" s="11"/>
+      <c r="D45" s="15">
+        <f t="shared" si="2"/>
+        <v>7.4999999999999991E-4</v>
+      </c>
+      <c r="E45" s="15"/>
+    </row>
+    <row r="46" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B46" s="11">
+        <f>B24</f>
+        <v>20000</v>
+      </c>
+      <c r="C46" s="11"/>
+      <c r="D46" s="15">
+        <f t="shared" si="2"/>
+        <v>9.999999999999998E-4</v>
+      </c>
+      <c r="E46" s="15"/>
+    </row>
+    <row r="47" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B47" s="11">
+        <f>B25</f>
+        <v>25000</v>
+      </c>
+      <c r="C47" s="11"/>
+      <c r="D47" s="15">
+        <f t="shared" si="2"/>
+        <v>1.2499999999999998E-3</v>
+      </c>
+      <c r="E47" s="15"/>
+    </row>
+    <row r="48" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B48" s="11">
+        <f>B26</f>
+        <v>30000</v>
+      </c>
+      <c r="C48" s="11"/>
+      <c r="D48" s="15">
+        <f t="shared" si="2"/>
+        <v>1.4999999999999998E-3</v>
+      </c>
+      <c r="E48" s="15"/>
+    </row>
+    <row r="49" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B49" s="11">
+        <f>B27</f>
+        <v>35000</v>
+      </c>
+      <c r="C49" s="11"/>
+      <c r="D49" s="15">
+        <f t="shared" si="2"/>
+        <v>1.7499999999999996E-3</v>
+      </c>
+      <c r="E49" s="15"/>
+    </row>
+    <row r="50" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B50" s="11">
+        <f>B28</f>
+        <v>40000</v>
+      </c>
+      <c r="C50" s="11"/>
+      <c r="D50" s="15">
+        <f t="shared" si="2"/>
+        <v>1.9999999999999996E-3</v>
+      </c>
+      <c r="E50" s="15"/>
+    </row>
+    <row r="52" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="I52" s="6"/>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="31">
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="D47:E47"/>
+    <mergeCell ref="D48:E48"/>
+    <mergeCell ref="D49:E49"/>
+    <mergeCell ref="D50:E50"/>
+    <mergeCell ref="D41:E41"/>
+    <mergeCell ref="D42:E42"/>
+    <mergeCell ref="D43:E43"/>
+    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="B46:C46"/>
+    <mergeCell ref="B47:C47"/>
+    <mergeCell ref="B48:C48"/>
+    <mergeCell ref="B49:C49"/>
+    <mergeCell ref="B50:C50"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="B43:C43"/>
+    <mergeCell ref="B44:C44"/>
+    <mergeCell ref="B45:C45"/>
+    <mergeCell ref="B40:E40"/>
+    <mergeCell ref="B39:E39"/>
+    <mergeCell ref="B32:E32"/>
+    <mergeCell ref="B31:E31"/>
+    <mergeCell ref="B33:C33"/>
     <mergeCell ref="B18:C18"/>
     <mergeCell ref="B16:G16"/>
     <mergeCell ref="E18:G18"/>

</xml_diff>

<commit_message>
se realizó el calculo de la diferencia relativa entre la deflexion teorica y la medida
</commit_message>
<xml_diff>
--- a/Analysis/Cálculos.xlsx
+++ b/Analysis/Cálculos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\david\Documents\Evaluacion 1 Herramientas\Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8678DB06-72F3-411F-A14D-A36F3E49729D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F9487C0-63B6-4C73-B2D6-E7FF0BDDDA95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="25">
   <si>
     <t>Carga [KN]</t>
   </si>
@@ -105,6 +105,12 @@
   </si>
   <si>
     <t>Delta_teo = (P*(L^3))/(48*E*I)</t>
+  </si>
+  <si>
+    <t>(|delta_medida-delta_Teo| / delta_teo ) * 100</t>
+  </si>
+  <si>
+    <t>Diferencia relativa (%)</t>
   </si>
 </sst>
 </file>
@@ -112,9 +118,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="201" formatCode="0.00000"/>
+    <numFmt numFmtId="164" formatCode="0.00000"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -124,6 +130,13 @@
     </font>
     <font>
       <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -213,10 +226,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -232,6 +246,27 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -241,30 +276,13 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="201" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="201" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Porcentaje" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -542,35 +560,35 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:J52"/>
+  <dimension ref="B2:J63"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="16.33203125" customWidth="1"/>
+    <col min="2" max="2" width="24.88671875" customWidth="1"/>
     <col min="3" max="3" width="23.21875" customWidth="1"/>
     <col min="5" max="5" width="30" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
-      <c r="G2" s="9"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="8"/>
-      <c r="E4" s="8" t="s">
+      <c r="C4" s="15"/>
+      <c r="E4" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="F4" s="8"/>
-      <c r="G4" s="8"/>
+      <c r="F4" s="15"/>
+      <c r="G4" s="15"/>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B5" s="1" t="s">
@@ -689,25 +707,25 @@
       </c>
     </row>
     <row r="16" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="C16" s="7"/>
-      <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="7"/>
-      <c r="G16" s="7"/>
+      <c r="C16" s="14"/>
+      <c r="D16" s="14"/>
+      <c r="E16" s="14"/>
+      <c r="F16" s="14"/>
+      <c r="G16" s="14"/>
     </row>
     <row r="18" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="7"/>
-      <c r="E18" s="7" t="s">
+      <c r="C18" s="14"/>
+      <c r="E18" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="F18" s="7"/>
-      <c r="G18" s="7"/>
+      <c r="F18" s="14"/>
+      <c r="G18" s="14"/>
       <c r="J18" s="6"/>
     </row>
     <row r="19" spans="2:10" x14ac:dyDescent="0.3">
@@ -751,7 +769,7 @@
         <f t="shared" si="0"/>
         <v>5000</v>
       </c>
-      <c r="C21" s="16">
+      <c r="C21" s="7">
         <f t="shared" si="1"/>
         <v>2.6000000000000003E-4</v>
       </c>
@@ -846,20 +864,20 @@
       </c>
     </row>
     <row r="31" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B31" s="10" t="s">
+      <c r="B31" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="C31" s="10"/>
-      <c r="D31" s="10"/>
-      <c r="E31" s="10"/>
+      <c r="C31" s="11"/>
+      <c r="D31" s="11"/>
+      <c r="E31" s="11"/>
     </row>
     <row r="32" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B32" s="10" t="s">
+      <c r="B32" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="C32" s="10"/>
-      <c r="D32" s="10"/>
-      <c r="E32" s="10"/>
+      <c r="C32" s="11"/>
+      <c r="D32" s="11"/>
+      <c r="E32" s="11"/>
     </row>
     <row r="33" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B33" s="12" t="s">
@@ -875,175 +893,260 @@
       </c>
     </row>
     <row r="39" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B39" s="14" t="s">
+      <c r="B39" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="C39" s="14"/>
-      <c r="D39" s="14"/>
-      <c r="E39" s="14"/>
+      <c r="C39" s="10"/>
+      <c r="D39" s="10"/>
+      <c r="E39" s="10"/>
     </row>
     <row r="40" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B40" s="14" t="s">
+      <c r="B40" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="C40" s="14"/>
-      <c r="D40" s="14"/>
-      <c r="E40" s="14"/>
+      <c r="C40" s="10"/>
+      <c r="D40" s="10"/>
+      <c r="E40" s="10"/>
     </row>
     <row r="41" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B41" s="11" t="s">
+      <c r="B41" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="C41" s="11"/>
-      <c r="D41" s="11" t="s">
+      <c r="C41" s="9"/>
+      <c r="D41" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="E41" s="11"/>
+      <c r="E41" s="9"/>
     </row>
     <row r="42" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B42" s="11">
-        <f>B20</f>
+      <c r="B42" s="9">
+        <f t="shared" ref="B42:B50" si="2">B20</f>
         <v>0</v>
       </c>
-      <c r="C42" s="11"/>
-      <c r="D42" s="11">
+      <c r="C42" s="9"/>
+      <c r="D42" s="9">
         <f>B42*(($G$19)^3)/48*$E$33*$G$22</f>
         <v>0</v>
       </c>
-      <c r="E42" s="11"/>
+      <c r="E42" s="9"/>
     </row>
     <row r="43" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B43" s="11">
-        <f>B21</f>
+      <c r="B43" s="9">
+        <f t="shared" si="2"/>
         <v>5000</v>
       </c>
-      <c r="C43" s="11"/>
-      <c r="D43" s="15">
+      <c r="C43" s="9"/>
+      <c r="D43" s="8">
         <f>B43*(($G$19)^3)/(48*$E$33*$G$22)</f>
         <v>2.4999999999999995E-4</v>
       </c>
-      <c r="E43" s="15"/>
+      <c r="E43" s="8"/>
     </row>
     <row r="44" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B44" s="11">
-        <f>B22</f>
+      <c r="B44" s="9">
+        <f t="shared" si="2"/>
         <v>10000</v>
       </c>
-      <c r="C44" s="11"/>
-      <c r="D44" s="15">
-        <f t="shared" ref="D44:D50" si="2">B44*(($G$19)^3)/(48*$E$33*$G$22)</f>
+      <c r="C44" s="9"/>
+      <c r="D44" s="8">
+        <f t="shared" ref="D44:D50" si="3">B44*(($G$19)^3)/(48*$E$33*$G$22)</f>
         <v>4.999999999999999E-4</v>
       </c>
-      <c r="E44" s="15"/>
+      <c r="E44" s="8"/>
     </row>
     <row r="45" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B45" s="11">
-        <f>B23</f>
+      <c r="B45" s="9">
+        <f t="shared" si="2"/>
         <v>15000</v>
       </c>
-      <c r="C45" s="11"/>
-      <c r="D45" s="15">
+      <c r="C45" s="9"/>
+      <c r="D45" s="8">
+        <f t="shared" si="3"/>
+        <v>7.4999999999999991E-4</v>
+      </c>
+      <c r="E45" s="8"/>
+    </row>
+    <row r="46" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B46" s="9">
         <f t="shared" si="2"/>
-        <v>7.4999999999999991E-4</v>
-      </c>
-      <c r="E45" s="15"/>
-    </row>
-    <row r="46" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B46" s="11">
-        <f>B24</f>
         <v>20000</v>
       </c>
-      <c r="C46" s="11"/>
-      <c r="D46" s="15">
+      <c r="C46" s="9"/>
+      <c r="D46" s="8">
+        <f t="shared" si="3"/>
+        <v>9.999999999999998E-4</v>
+      </c>
+      <c r="E46" s="8"/>
+    </row>
+    <row r="47" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B47" s="9">
         <f t="shared" si="2"/>
-        <v>9.999999999999998E-4</v>
-      </c>
-      <c r="E46" s="15"/>
-    </row>
-    <row r="47" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B47" s="11">
-        <f>B25</f>
         <v>25000</v>
       </c>
-      <c r="C47" s="11"/>
-      <c r="D47" s="15">
+      <c r="C47" s="9"/>
+      <c r="D47" s="8">
+        <f t="shared" si="3"/>
+        <v>1.2499999999999998E-3</v>
+      </c>
+      <c r="E47" s="8"/>
+    </row>
+    <row r="48" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B48" s="9">
         <f t="shared" si="2"/>
-        <v>1.2499999999999998E-3</v>
-      </c>
-      <c r="E47" s="15"/>
-    </row>
-    <row r="48" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B48" s="11">
-        <f>B26</f>
         <v>30000</v>
       </c>
-      <c r="C48" s="11"/>
-      <c r="D48" s="15">
+      <c r="C48" s="9"/>
+      <c r="D48" s="8">
+        <f t="shared" si="3"/>
+        <v>1.4999999999999998E-3</v>
+      </c>
+      <c r="E48" s="8"/>
+    </row>
+    <row r="49" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B49" s="9">
         <f t="shared" si="2"/>
-        <v>1.4999999999999998E-3</v>
-      </c>
-      <c r="E48" s="15"/>
-    </row>
-    <row r="49" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B49" s="11">
-        <f>B27</f>
         <v>35000</v>
       </c>
-      <c r="C49" s="11"/>
-      <c r="D49" s="15">
+      <c r="C49" s="9"/>
+      <c r="D49" s="8">
+        <f t="shared" si="3"/>
+        <v>1.7499999999999996E-3</v>
+      </c>
+      <c r="E49" s="8"/>
+    </row>
+    <row r="50" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B50" s="9">
         <f t="shared" si="2"/>
-        <v>1.7499999999999996E-3</v>
-      </c>
-      <c r="E49" s="15"/>
-    </row>
-    <row r="50" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B50" s="11">
-        <f>B28</f>
         <v>40000</v>
       </c>
-      <c r="C50" s="11"/>
-      <c r="D50" s="15">
-        <f t="shared" si="2"/>
+      <c r="C50" s="9"/>
+      <c r="D50" s="8">
+        <f t="shared" si="3"/>
         <v>1.9999999999999996E-3</v>
       </c>
-      <c r="E50" s="15"/>
+      <c r="E50" s="8"/>
     </row>
     <row r="52" spans="2:9" x14ac:dyDescent="0.3">
       <c r="I52" s="6"/>
     </row>
+    <row r="53" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B53" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="C53" s="10"/>
+    </row>
+    <row r="54" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B54" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="C54" s="10"/>
+    </row>
+    <row r="55" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B55" s="17">
+        <v>0</v>
+      </c>
+      <c r="C55" s="17"/>
+    </row>
+    <row r="56" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B56" s="17">
+        <f>(C21-D43)/D43</f>
+        <v>4.0000000000000327E-2</v>
+      </c>
+      <c r="C56" s="17"/>
+    </row>
+    <row r="57" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B57" s="17">
+        <f>(C22-D44)/D44</f>
+        <v>2.1684043449710094E-16</v>
+      </c>
+      <c r="C57" s="17"/>
+    </row>
+    <row r="58" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B58" s="17">
+        <f>(C23-D45)/D45</f>
+        <v>1.3333333333333515E-2</v>
+      </c>
+      <c r="C58" s="17"/>
+    </row>
+    <row r="59" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B59" s="17">
+        <f>(C24-D46)/D46</f>
+        <v>1.0000000000000245E-2</v>
+      </c>
+      <c r="C59" s="17"/>
+    </row>
+    <row r="60" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B60" s="17">
+        <f>(C25-D47)/D47</f>
+        <v>2.400000000000024E-2</v>
+      </c>
+      <c r="C60" s="17"/>
+    </row>
+    <row r="61" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B61" s="17">
+        <f>(C26-D48)/D48</f>
+        <v>2.6666666666666883E-2</v>
+      </c>
+      <c r="C61" s="17"/>
+    </row>
+    <row r="62" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B62" s="17">
+        <f>(C27-D49)/D49</f>
+        <v>1.142857142857171E-2</v>
+      </c>
+      <c r="C62" s="17"/>
+    </row>
+    <row r="63" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B63" s="17">
+        <f>(C28-D50)/D50</f>
+        <v>2.5000000000000071E-2</v>
+      </c>
+      <c r="C63" s="17"/>
+    </row>
   </sheetData>
-  <mergeCells count="31">
-    <mergeCell ref="D46:E46"/>
-    <mergeCell ref="D47:E47"/>
-    <mergeCell ref="D48:E48"/>
-    <mergeCell ref="D49:E49"/>
-    <mergeCell ref="D50:E50"/>
-    <mergeCell ref="D41:E41"/>
-    <mergeCell ref="D42:E42"/>
-    <mergeCell ref="D43:E43"/>
-    <mergeCell ref="D44:E44"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="B46:C46"/>
-    <mergeCell ref="B47:C47"/>
-    <mergeCell ref="B48:C48"/>
-    <mergeCell ref="B49:C49"/>
-    <mergeCell ref="B50:C50"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B42:C42"/>
-    <mergeCell ref="B43:C43"/>
-    <mergeCell ref="B44:C44"/>
-    <mergeCell ref="B45:C45"/>
-    <mergeCell ref="B40:E40"/>
-    <mergeCell ref="B39:E39"/>
-    <mergeCell ref="B32:E32"/>
-    <mergeCell ref="B31:E31"/>
-    <mergeCell ref="B33:C33"/>
+  <mergeCells count="42">
+    <mergeCell ref="B54:C54"/>
+    <mergeCell ref="B55:C55"/>
+    <mergeCell ref="B56:C56"/>
+    <mergeCell ref="B57:C57"/>
+    <mergeCell ref="B63:C63"/>
+    <mergeCell ref="B58:C58"/>
+    <mergeCell ref="B59:C59"/>
+    <mergeCell ref="B60:C60"/>
+    <mergeCell ref="B61:C61"/>
+    <mergeCell ref="B62:C62"/>
+    <mergeCell ref="B53:C53"/>
     <mergeCell ref="B18:C18"/>
     <mergeCell ref="B16:G16"/>
     <mergeCell ref="E18:G18"/>
     <mergeCell ref="E4:G4"/>
     <mergeCell ref="B2:G2"/>
     <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B40:E40"/>
+    <mergeCell ref="B39:E39"/>
+    <mergeCell ref="B32:E32"/>
+    <mergeCell ref="B31:E31"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="B43:C43"/>
+    <mergeCell ref="B44:C44"/>
+    <mergeCell ref="B45:C45"/>
+    <mergeCell ref="B46:C46"/>
+    <mergeCell ref="B47:C47"/>
+    <mergeCell ref="B48:C48"/>
+    <mergeCell ref="B49:C49"/>
+    <mergeCell ref="B50:C50"/>
+    <mergeCell ref="D41:E41"/>
+    <mergeCell ref="D42:E42"/>
+    <mergeCell ref="D43:E43"/>
+    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="D47:E47"/>
+    <mergeCell ref="D48:E48"/>
+    <mergeCell ref="D49:E49"/>
+    <mergeCell ref="D50:E50"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
se añadio nota tecnica junto a sus archivos correspondientes
</commit_message>
<xml_diff>
--- a/Analysis/Cálculos.xlsx
+++ b/Analysis/Cálculos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\david\Documents\Evaluacion 1 Herramientas\Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F9487C0-63B6-4C73-B2D6-E7FF0BDDDA95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DFDCF36-5A8F-4F82-A7C8-ED24D34DB157}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="31">
   <si>
     <t>Carga [KN]</t>
   </si>
@@ -111,14 +111,33 @@
   </si>
   <si>
     <t>Diferencia relativa (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verificacion de linealidad </t>
+  </si>
+  <si>
+    <t>delta/P</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>delta [mm]</t>
+  </si>
+  <si>
+    <t>P [KN]</t>
+  </si>
+  <si>
+    <t>delta/p [mm/KN]</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.00000"/>
+    <numFmt numFmtId="166" formatCode="0.000"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -144,7 +163,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -172,6 +191,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -230,7 +255,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -249,22 +274,10 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -276,7 +289,23 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -295,6 +324,1363 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="es-MX"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-CL"/>
+              <a:t>Carga</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="es-CL" baseline="0"/>
+              <a:t>-deflexión: Experimental vs teórica </a:t>
+            </a:r>
+            <a:endParaRPr lang="es-CL"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-CL"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Deflexión medida</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Hoja1!$B$20:$B$28</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>5000</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>10000</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>15000</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>20000</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>25000</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>30000</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>35000</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>40000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Hoja1!$C$20:$C$28</c:f>
+              <c:numCache>
+                <c:formatCode>0.00000</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0" formatCode="General">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2.6000000000000003E-4</c:v>
+                </c:pt>
+                <c:pt idx="2" formatCode="General">
+                  <c:v>5.0000000000000001E-4</c:v>
+                </c:pt>
+                <c:pt idx="3" formatCode="General">
+                  <c:v>7.6000000000000004E-4</c:v>
+                </c:pt>
+                <c:pt idx="4" formatCode="General">
+                  <c:v>1.01E-3</c:v>
+                </c:pt>
+                <c:pt idx="5" formatCode="General">
+                  <c:v>1.2800000000000001E-3</c:v>
+                </c:pt>
+                <c:pt idx="6" formatCode="General">
+                  <c:v>1.5400000000000001E-3</c:v>
+                </c:pt>
+                <c:pt idx="7" formatCode="General">
+                  <c:v>1.7700000000000001E-3</c:v>
+                </c:pt>
+                <c:pt idx="8" formatCode="General">
+                  <c:v>2.0499999999999997E-3</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-F592-41C2-A237-52E35051B8E8}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Deflexión teórica</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Hoja1!$B$20:$B$28</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>5000</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>10000</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>15000</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>20000</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>25000</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>30000</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>35000</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>40000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Hoja1!$D$42:$D$50</c:f>
+              <c:numCache>
+                <c:formatCode>0.00000</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0" formatCode="General">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2.4999999999999995E-4</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4.999999999999999E-4</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>7.4999999999999991E-4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>9.999999999999998E-4</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1.2499999999999998E-3</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1.4999999999999998E-3</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1.7499999999999996E-3</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.9999999999999996E-3</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-F592-41C2-A237-52E35051B8E8}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Hoja1!$E$41</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent3"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Hoja1!$B$20:$B$28</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>5000</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>10000</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>15000</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>20000</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>25000</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>30000</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>35000</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>40000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Hoja1!$E$42:$E$50</c:f>
+              <c:numCache>
+                <c:formatCode>0.00000</c:formatCode>
+                <c:ptCount val="9"/>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-F592-41C2-A237-52E35051B8E8}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="835704800"/>
+        <c:axId val="831187856"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="835704800"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="40000"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="es-CL"/>
+                  <a:t>Carga</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="es-CL" baseline="0"/>
+                  <a:t> [N]</a:t>
+                </a:r>
+                <a:endParaRPr lang="es-CL"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="es-CL"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="es-CL"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="831187856"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="831187856"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="2.2000000000000006E-3"/>
+          <c:min val="0"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="es-CL"/>
+                  <a:t>Deflexión</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="es-CL" baseline="0"/>
+                  <a:t> [m]</a:t>
+                </a:r>
+                <a:endParaRPr lang="es-CL"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="es-CL"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="es-CL"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="835704800"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:legendEntry>
+        <c:idx val="2"/>
+        <c:delete val="1"/>
+      </c:legendEntry>
+      <c:legendEntry>
+        <c:idx val="3"/>
+        <c:delete val="1"/>
+      </c:legendEntry>
+      <c:legendEntry>
+        <c:idx val="4"/>
+        <c:delete val="1"/>
+      </c:legendEntry>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-CL"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="es-CL"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>10990</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>57151</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>603738</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>99647</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Gráfico 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{153F1BF4-A448-1A2F-10A1-F1F3CF4D1378}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -560,35 +1946,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:J63"/>
+  <dimension ref="B2:Q76"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="24.88671875" customWidth="1"/>
     <col min="3" max="3" width="23.21875" customWidth="1"/>
+    <col min="4" max="4" width="14.88671875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="30" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B2" s="16" t="s">
+      <c r="B2" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B4" s="15" t="s">
+      <c r="B4" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="15"/>
-      <c r="E4" s="15" t="s">
+      <c r="C4" s="11"/>
+      <c r="E4" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="F4" s="15"/>
-      <c r="G4" s="15"/>
+      <c r="F4" s="11"/>
+      <c r="G4" s="11"/>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B5" s="1" t="s">
@@ -707,25 +2094,25 @@
       </c>
     </row>
     <row r="16" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B16" s="14" t="s">
+      <c r="B16" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="C16" s="14"/>
-      <c r="D16" s="14"/>
-      <c r="E16" s="14"/>
-      <c r="F16" s="14"/>
-      <c r="G16" s="14"/>
+      <c r="C16" s="10"/>
+      <c r="D16" s="10"/>
+      <c r="E16" s="10"/>
+      <c r="F16" s="10"/>
+      <c r="G16" s="10"/>
     </row>
     <row r="18" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B18" s="14" t="s">
+      <c r="B18" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="14"/>
-      <c r="E18" s="14" t="s">
+      <c r="C18" s="10"/>
+      <c r="E18" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="F18" s="14"/>
-      <c r="G18" s="14"/>
+      <c r="F18" s="10"/>
+      <c r="G18" s="10"/>
       <c r="J18" s="6"/>
     </row>
     <row r="19" spans="2:10" x14ac:dyDescent="0.3">
@@ -864,26 +2251,26 @@
       </c>
     </row>
     <row r="31" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B31" s="11" t="s">
+      <c r="B31" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="C31" s="11"/>
-      <c r="D31" s="11"/>
-      <c r="E31" s="11"/>
+      <c r="C31" s="13"/>
+      <c r="D31" s="13"/>
+      <c r="E31" s="13"/>
     </row>
     <row r="32" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B32" s="11" t="s">
+      <c r="B32" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="C32" s="11"/>
-      <c r="D32" s="11"/>
-      <c r="E32" s="11"/>
-    </row>
-    <row r="33" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B33" s="12" t="s">
+      <c r="C32" s="13"/>
+      <c r="D32" s="13"/>
+      <c r="E32" s="13"/>
+    </row>
+    <row r="33" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="B33" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="C33" s="13"/>
+      <c r="C33" s="15"/>
       <c r="D33" s="3" t="s">
         <v>19</v>
       </c>
@@ -891,235 +2278,364 @@
         <f>(G20*(G21)^3)/12</f>
         <v>1.0666666666666669E-3</v>
       </c>
-    </row>
-    <row r="39" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B39" s="10" t="s">
+      <c r="Q33" s="6"/>
+    </row>
+    <row r="39" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="B39" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="C39" s="10"/>
-      <c r="D39" s="10"/>
-      <c r="E39" s="10"/>
-    </row>
-    <row r="40" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B40" s="10" t="s">
+      <c r="C39" s="8"/>
+      <c r="D39" s="8"/>
+      <c r="E39" s="8"/>
+    </row>
+    <row r="40" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="B40" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="C40" s="10"/>
-      <c r="D40" s="10"/>
-      <c r="E40" s="10"/>
-    </row>
-    <row r="41" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B41" s="9" t="s">
+      <c r="C40" s="8"/>
+      <c r="D40" s="8"/>
+      <c r="E40" s="8"/>
+    </row>
+    <row r="41" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="B41" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="C41" s="9"/>
-      <c r="D41" s="9" t="s">
+      <c r="C41" s="16"/>
+      <c r="D41" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="E41" s="9"/>
-    </row>
-    <row r="42" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B42" s="9">
+      <c r="E41" s="16"/>
+    </row>
+    <row r="42" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="B42" s="16">
         <f t="shared" ref="B42:B50" si="2">B20</f>
         <v>0</v>
       </c>
-      <c r="C42" s="9"/>
-      <c r="D42" s="9">
+      <c r="C42" s="16"/>
+      <c r="D42" s="16">
         <f>B42*(($G$19)^3)/48*$E$33*$G$22</f>
         <v>0</v>
       </c>
-      <c r="E42" s="9"/>
-    </row>
-    <row r="43" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B43" s="9">
+      <c r="E42" s="16"/>
+    </row>
+    <row r="43" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="B43" s="16">
         <f t="shared" si="2"/>
         <v>5000</v>
       </c>
-      <c r="C43" s="9"/>
-      <c r="D43" s="8">
+      <c r="C43" s="16"/>
+      <c r="D43" s="17">
         <f>B43*(($G$19)^3)/(48*$E$33*$G$22)</f>
         <v>2.4999999999999995E-4</v>
       </c>
-      <c r="E43" s="8"/>
-    </row>
-    <row r="44" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B44" s="9">
+      <c r="E43" s="17"/>
+    </row>
+    <row r="44" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="B44" s="16">
         <f t="shared" si="2"/>
         <v>10000</v>
       </c>
-      <c r="C44" s="9"/>
-      <c r="D44" s="8">
+      <c r="C44" s="16"/>
+      <c r="D44" s="17">
         <f t="shared" ref="D44:D50" si="3">B44*(($G$19)^3)/(48*$E$33*$G$22)</f>
         <v>4.999999999999999E-4</v>
       </c>
-      <c r="E44" s="8"/>
-    </row>
-    <row r="45" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B45" s="9">
+      <c r="E44" s="17"/>
+    </row>
+    <row r="45" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="B45" s="16">
         <f t="shared" si="2"/>
         <v>15000</v>
       </c>
-      <c r="C45" s="9"/>
-      <c r="D45" s="8">
+      <c r="C45" s="16"/>
+      <c r="D45" s="17">
         <f t="shared" si="3"/>
         <v>7.4999999999999991E-4</v>
       </c>
-      <c r="E45" s="8"/>
-    </row>
-    <row r="46" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B46" s="9">
+      <c r="E45" s="17"/>
+    </row>
+    <row r="46" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="B46" s="16">
         <f t="shared" si="2"/>
         <v>20000</v>
       </c>
-      <c r="C46" s="9"/>
-      <c r="D46" s="8">
+      <c r="C46" s="16"/>
+      <c r="D46" s="17">
         <f t="shared" si="3"/>
         <v>9.999999999999998E-4</v>
       </c>
-      <c r="E46" s="8"/>
-    </row>
-    <row r="47" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B47" s="9">
+      <c r="E46" s="17"/>
+    </row>
+    <row r="47" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="B47" s="16">
         <f t="shared" si="2"/>
         <v>25000</v>
       </c>
-      <c r="C47" s="9"/>
-      <c r="D47" s="8">
+      <c r="C47" s="16"/>
+      <c r="D47" s="17">
         <f t="shared" si="3"/>
         <v>1.2499999999999998E-3</v>
       </c>
-      <c r="E47" s="8"/>
-    </row>
-    <row r="48" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B48" s="9">
+      <c r="E47" s="17"/>
+    </row>
+    <row r="48" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="B48" s="16">
         <f t="shared" si="2"/>
         <v>30000</v>
       </c>
-      <c r="C48" s="9"/>
-      <c r="D48" s="8">
+      <c r="C48" s="16"/>
+      <c r="D48" s="17">
         <f t="shared" si="3"/>
         <v>1.4999999999999998E-3</v>
       </c>
-      <c r="E48" s="8"/>
+      <c r="E48" s="17"/>
     </row>
     <row r="49" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B49" s="9">
+      <c r="B49" s="16">
         <f t="shared" si="2"/>
         <v>35000</v>
       </c>
-      <c r="C49" s="9"/>
-      <c r="D49" s="8">
+      <c r="C49" s="16"/>
+      <c r="D49" s="17">
         <f t="shared" si="3"/>
         <v>1.7499999999999996E-3</v>
       </c>
-      <c r="E49" s="8"/>
+      <c r="E49" s="17"/>
     </row>
     <row r="50" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B50" s="9">
+      <c r="B50" s="16">
         <f t="shared" si="2"/>
         <v>40000</v>
       </c>
-      <c r="C50" s="9"/>
-      <c r="D50" s="8">
+      <c r="C50" s="16"/>
+      <c r="D50" s="17">
         <f t="shared" si="3"/>
         <v>1.9999999999999996E-3</v>
       </c>
-      <c r="E50" s="8"/>
+      <c r="E50" s="17"/>
     </row>
     <row r="52" spans="2:9" x14ac:dyDescent="0.3">
       <c r="I52" s="6"/>
     </row>
     <row r="53" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B53" s="10" t="s">
+      <c r="B53" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="C53" s="10"/>
+      <c r="C53" s="8"/>
     </row>
     <row r="54" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B54" s="10" t="s">
+      <c r="B54" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="C54" s="10"/>
+      <c r="C54" s="8"/>
     </row>
     <row r="55" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B55" s="17">
+      <c r="B55" s="9">
         <v>0</v>
       </c>
-      <c r="C55" s="17"/>
+      <c r="C55" s="9"/>
     </row>
     <row r="56" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B56" s="17">
-        <f>(C21-D43)/D43</f>
+      <c r="B56" s="9">
+        <f t="shared" ref="B56:B63" si="4">(C21-D43)/D43</f>
         <v>4.0000000000000327E-2</v>
       </c>
-      <c r="C56" s="17"/>
+      <c r="C56" s="9"/>
     </row>
     <row r="57" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B57" s="17">
-        <f>(C22-D44)/D44</f>
+      <c r="B57" s="9">
+        <f t="shared" si="4"/>
         <v>2.1684043449710094E-16</v>
       </c>
-      <c r="C57" s="17"/>
+      <c r="C57" s="9"/>
     </row>
     <row r="58" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B58" s="17">
-        <f>(C23-D45)/D45</f>
+      <c r="B58" s="9">
+        <f t="shared" si="4"/>
         <v>1.3333333333333515E-2</v>
       </c>
-      <c r="C58" s="17"/>
+      <c r="C58" s="9"/>
     </row>
     <row r="59" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B59" s="17">
-        <f>(C24-D46)/D46</f>
+      <c r="B59" s="9">
+        <f t="shared" si="4"/>
         <v>1.0000000000000245E-2</v>
       </c>
-      <c r="C59" s="17"/>
+      <c r="C59" s="9"/>
     </row>
     <row r="60" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B60" s="17">
-        <f>(C25-D47)/D47</f>
+      <c r="B60" s="9">
+        <f t="shared" si="4"/>
         <v>2.400000000000024E-2</v>
       </c>
-      <c r="C60" s="17"/>
+      <c r="C60" s="9"/>
     </row>
     <row r="61" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B61" s="17">
-        <f>(C26-D48)/D48</f>
+      <c r="B61" s="9">
+        <f t="shared" si="4"/>
         <v>2.6666666666666883E-2</v>
       </c>
-      <c r="C61" s="17"/>
+      <c r="C61" s="9"/>
     </row>
     <row r="62" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B62" s="17">
-        <f>(C27-D49)/D49</f>
+      <c r="B62" s="9">
+        <f t="shared" si="4"/>
         <v>1.142857142857171E-2</v>
       </c>
-      <c r="C62" s="17"/>
+      <c r="C62" s="9"/>
     </row>
     <row r="63" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B63" s="17">
-        <f>(C28-D50)/D50</f>
+      <c r="B63" s="9">
+        <f t="shared" si="4"/>
         <v>2.5000000000000071E-2</v>
       </c>
-      <c r="C63" s="17"/>
+      <c r="C63" s="9"/>
+    </row>
+    <row r="65" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B65" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="C65" s="13"/>
+      <c r="D65" s="13"/>
+    </row>
+    <row r="66" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B66" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="C66" s="13"/>
+      <c r="D66" s="13"/>
+    </row>
+    <row r="67" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B67" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="C67" s="19" t="s">
+        <v>29</v>
+      </c>
+      <c r="D67" s="19" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="68" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B68" s="3">
+        <v>0</v>
+      </c>
+      <c r="C68" s="4">
+        <v>0</v>
+      </c>
+      <c r="D68" s="4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="69" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B69" s="3">
+        <v>0.26</v>
+      </c>
+      <c r="C69" s="3">
+        <v>5</v>
+      </c>
+      <c r="D69" s="18">
+        <f>B69/C69</f>
+        <v>5.2000000000000005E-2</v>
+      </c>
+    </row>
+    <row r="70" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B70" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="C70" s="3">
+        <v>10</v>
+      </c>
+      <c r="D70" s="18">
+        <f t="shared" ref="D70:D76" si="5">B70/C70</f>
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="71" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B71" s="3">
+        <v>0.76</v>
+      </c>
+      <c r="C71" s="3">
+        <v>15</v>
+      </c>
+      <c r="D71" s="18">
+        <f t="shared" si="5"/>
+        <v>5.0666666666666665E-2</v>
+      </c>
+    </row>
+    <row r="72" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B72" s="3">
+        <v>1.01</v>
+      </c>
+      <c r="C72" s="3">
+        <v>20</v>
+      </c>
+      <c r="D72" s="18">
+        <f t="shared" si="5"/>
+        <v>5.0500000000000003E-2</v>
+      </c>
+    </row>
+    <row r="73" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B73" s="3">
+        <v>1.28</v>
+      </c>
+      <c r="C73" s="3">
+        <v>25</v>
+      </c>
+      <c r="D73" s="18">
+        <f t="shared" si="5"/>
+        <v>5.1200000000000002E-2</v>
+      </c>
+    </row>
+    <row r="74" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B74" s="3">
+        <v>1.54</v>
+      </c>
+      <c r="C74" s="3">
+        <v>30</v>
+      </c>
+      <c r="D74" s="18">
+        <f t="shared" si="5"/>
+        <v>5.1333333333333335E-2</v>
+      </c>
+    </row>
+    <row r="75" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B75" s="3">
+        <v>1.77</v>
+      </c>
+      <c r="C75" s="3">
+        <v>35</v>
+      </c>
+      <c r="D75" s="18">
+        <f t="shared" si="5"/>
+        <v>5.0571428571428573E-2</v>
+      </c>
+    </row>
+    <row r="76" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B76" s="3">
+        <v>2.0499999999999998</v>
+      </c>
+      <c r="C76" s="3">
+        <v>40</v>
+      </c>
+      <c r="D76" s="18">
+        <f t="shared" si="5"/>
+        <v>5.1249999999999997E-2</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="42">
-    <mergeCell ref="B54:C54"/>
-    <mergeCell ref="B55:C55"/>
-    <mergeCell ref="B56:C56"/>
-    <mergeCell ref="B57:C57"/>
-    <mergeCell ref="B63:C63"/>
-    <mergeCell ref="B58:C58"/>
-    <mergeCell ref="B59:C59"/>
-    <mergeCell ref="B60:C60"/>
-    <mergeCell ref="B61:C61"/>
-    <mergeCell ref="B62:C62"/>
-    <mergeCell ref="B53:C53"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B16:G16"/>
-    <mergeCell ref="E18:G18"/>
-    <mergeCell ref="E4:G4"/>
+  <mergeCells count="44">
+    <mergeCell ref="B65:D65"/>
+    <mergeCell ref="B66:D66"/>
+    <mergeCell ref="D47:E47"/>
+    <mergeCell ref="D48:E48"/>
+    <mergeCell ref="D49:E49"/>
+    <mergeCell ref="D50:E50"/>
+    <mergeCell ref="D42:E42"/>
+    <mergeCell ref="D43:E43"/>
+    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="D46:E46"/>
     <mergeCell ref="B2:G2"/>
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="B40:E40"/>
@@ -1127,6 +2643,11 @@
     <mergeCell ref="B32:E32"/>
     <mergeCell ref="B31:E31"/>
     <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B53:C53"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B16:G16"/>
+    <mergeCell ref="E18:G18"/>
+    <mergeCell ref="E4:G4"/>
     <mergeCell ref="B41:C41"/>
     <mergeCell ref="B42:C42"/>
     <mergeCell ref="B43:C43"/>
@@ -1138,17 +2659,19 @@
     <mergeCell ref="B49:C49"/>
     <mergeCell ref="B50:C50"/>
     <mergeCell ref="D41:E41"/>
-    <mergeCell ref="D42:E42"/>
-    <mergeCell ref="D43:E43"/>
-    <mergeCell ref="D44:E44"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="D46:E46"/>
-    <mergeCell ref="D47:E47"/>
-    <mergeCell ref="D48:E48"/>
-    <mergeCell ref="D49:E49"/>
-    <mergeCell ref="D50:E50"/>
+    <mergeCell ref="B54:C54"/>
+    <mergeCell ref="B55:C55"/>
+    <mergeCell ref="B56:C56"/>
+    <mergeCell ref="B57:C57"/>
+    <mergeCell ref="B63:C63"/>
+    <mergeCell ref="B58:C58"/>
+    <mergeCell ref="B59:C59"/>
+    <mergeCell ref="B60:C60"/>
+    <mergeCell ref="B61:C61"/>
+    <mergeCell ref="B62:C62"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
se actualizaron ciertos cálculos en excel
</commit_message>
<xml_diff>
--- a/Analysis/Cálculos.xlsx
+++ b/Analysis/Cálculos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\david\Documents\Evaluacion 1 Herramientas\Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DFDCF36-5A8F-4F82-A7C8-ED24D34DB157}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F31B3170-A296-4008-8D71-627E89142D6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="33">
   <si>
     <t>Carga [KN]</t>
   </si>
@@ -129,6 +129,12 @@
   </si>
   <si>
     <t>delta/p [mm/KN]</t>
+  </si>
+  <si>
+    <t>Delta_teo [mm]</t>
+  </si>
+  <si>
+    <t>Carga (P) [KN]</t>
   </si>
 </sst>
 </file>
@@ -137,7 +143,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.00000"/>
-    <numFmt numFmtId="166" formatCode="0.000"/>
+    <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -274,22 +280,26 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
@@ -298,14 +308,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1646,16 +1652,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>10990</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>57151</xdr:rowOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>560077</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>23534</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>603738</xdr:colOff>
-      <xdr:row>41</xdr:row>
-      <xdr:rowOff>99647</xdr:rowOff>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>155502</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>66030</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1957,25 +1963,25 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="11"/>
-      <c r="E4" s="11" t="s">
+      <c r="C4" s="14"/>
+      <c r="E4" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="F4" s="11"/>
-      <c r="G4" s="11"/>
+      <c r="F4" s="14"/>
+      <c r="G4" s="14"/>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B5" s="1" t="s">
@@ -2094,25 +2100,25 @@
       </c>
     </row>
     <row r="16" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B16" s="10" t="s">
+      <c r="B16" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="C16" s="10"/>
-      <c r="D16" s="10"/>
-      <c r="E16" s="10"/>
-      <c r="F16" s="10"/>
-      <c r="G16" s="10"/>
+      <c r="C16" s="18"/>
+      <c r="D16" s="18"/>
+      <c r="E16" s="18"/>
+      <c r="F16" s="18"/>
+      <c r="G16" s="18"/>
     </row>
     <row r="18" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B18" s="10" t="s">
+      <c r="B18" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="10"/>
-      <c r="E18" s="10" t="s">
+      <c r="C18" s="18"/>
+      <c r="E18" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="F18" s="10"/>
-      <c r="G18" s="10"/>
+      <c r="F18" s="18"/>
+      <c r="G18" s="18"/>
       <c r="J18" s="6"/>
     </row>
     <row r="19" spans="2:10" x14ac:dyDescent="0.3">
@@ -2251,26 +2257,26 @@
       </c>
     </row>
     <row r="31" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B31" s="13" t="s">
+      <c r="B31" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="C31" s="13"/>
-      <c r="D31" s="13"/>
-      <c r="E31" s="13"/>
+      <c r="C31" s="10"/>
+      <c r="D31" s="10"/>
+      <c r="E31" s="10"/>
     </row>
     <row r="32" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B32" s="13" t="s">
+      <c r="B32" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="C32" s="13"/>
-      <c r="D32" s="13"/>
-      <c r="E32" s="13"/>
+      <c r="C32" s="10"/>
+      <c r="D32" s="10"/>
+      <c r="E32" s="10"/>
     </row>
     <row r="33" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B33" s="14" t="s">
+      <c r="B33" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="C33" s="15"/>
+      <c r="C33" s="17"/>
       <c r="D33" s="3" t="s">
         <v>19</v>
       </c>
@@ -2281,238 +2287,349 @@
       <c r="Q33" s="6"/>
     </row>
     <row r="39" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B39" s="8" t="s">
+      <c r="B39" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="C39" s="8"/>
-      <c r="D39" s="8"/>
-      <c r="E39" s="8"/>
+      <c r="C39" s="15"/>
+      <c r="D39" s="15"/>
+      <c r="E39" s="15"/>
+      <c r="G39" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="H39" s="15"/>
+      <c r="I39" s="15"/>
+      <c r="J39" s="15"/>
     </row>
     <row r="40" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B40" s="8" t="s">
+      <c r="B40" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="C40" s="8"/>
-      <c r="D40" s="8"/>
-      <c r="E40" s="8"/>
+      <c r="C40" s="15"/>
+      <c r="D40" s="15"/>
+      <c r="E40" s="15"/>
+      <c r="G40" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="H40" s="15"/>
+      <c r="I40" s="15"/>
+      <c r="J40" s="15"/>
     </row>
     <row r="41" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B41" s="16" t="s">
+      <c r="B41" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="C41" s="16"/>
-      <c r="D41" s="16" t="s">
+      <c r="C41" s="12"/>
+      <c r="D41" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="E41" s="16"/>
+      <c r="E41" s="12"/>
+      <c r="G41" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="H41" s="12"/>
+      <c r="I41" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="J41" s="12"/>
     </row>
     <row r="42" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B42" s="16">
+      <c r="B42" s="12">
         <f t="shared" ref="B42:B50" si="2">B20</f>
         <v>0</v>
       </c>
-      <c r="C42" s="16"/>
-      <c r="D42" s="16">
+      <c r="C42" s="12"/>
+      <c r="D42" s="12">
         <f>B42*(($G$19)^3)/48*$E$33*$G$22</f>
         <v>0</v>
       </c>
-      <c r="E42" s="16"/>
+      <c r="E42" s="12"/>
+      <c r="G42" s="12">
+        <f>B42/1000</f>
+        <v>0</v>
+      </c>
+      <c r="H42" s="12"/>
+      <c r="I42" s="12">
+        <f>D42*1000</f>
+        <v>0</v>
+      </c>
+      <c r="J42" s="12"/>
     </row>
     <row r="43" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B43" s="16">
+      <c r="B43" s="12">
         <f t="shared" si="2"/>
         <v>5000</v>
       </c>
-      <c r="C43" s="16"/>
-      <c r="D43" s="17">
+      <c r="C43" s="12"/>
+      <c r="D43" s="11">
         <f>B43*(($G$19)^3)/(48*$E$33*$G$22)</f>
         <v>2.4999999999999995E-4</v>
       </c>
-      <c r="E43" s="17"/>
+      <c r="E43" s="11"/>
+      <c r="G43" s="12">
+        <f t="shared" ref="G43:G50" si="3">B43/1000</f>
+        <v>5</v>
+      </c>
+      <c r="H43" s="12"/>
+      <c r="I43" s="12">
+        <f t="shared" ref="I43:I50" si="4">D43*1000</f>
+        <v>0.24999999999999994</v>
+      </c>
+      <c r="J43" s="12"/>
     </row>
     <row r="44" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B44" s="16">
+      <c r="B44" s="12">
         <f t="shared" si="2"/>
         <v>10000</v>
       </c>
-      <c r="C44" s="16"/>
-      <c r="D44" s="17">
-        <f t="shared" ref="D44:D50" si="3">B44*(($G$19)^3)/(48*$E$33*$G$22)</f>
+      <c r="C44" s="12"/>
+      <c r="D44" s="11">
+        <f t="shared" ref="D44:D50" si="5">B44*(($G$19)^3)/(48*$E$33*$G$22)</f>
         <v>4.999999999999999E-4</v>
       </c>
-      <c r="E44" s="17"/>
+      <c r="E44" s="11"/>
+      <c r="G44" s="12">
+        <f t="shared" si="3"/>
+        <v>10</v>
+      </c>
+      <c r="H44" s="12"/>
+      <c r="I44" s="12">
+        <f t="shared" si="4"/>
+        <v>0.49999999999999989</v>
+      </c>
+      <c r="J44" s="12"/>
     </row>
     <row r="45" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B45" s="16">
+      <c r="B45" s="12">
         <f t="shared" si="2"/>
         <v>15000</v>
       </c>
-      <c r="C45" s="16"/>
-      <c r="D45" s="17">
+      <c r="C45" s="12"/>
+      <c r="D45" s="11">
+        <f t="shared" si="5"/>
+        <v>7.4999999999999991E-4</v>
+      </c>
+      <c r="E45" s="11"/>
+      <c r="G45" s="12">
         <f t="shared" si="3"/>
-        <v>7.4999999999999991E-4</v>
-      </c>
-      <c r="E45" s="17"/>
+        <v>15</v>
+      </c>
+      <c r="H45" s="12"/>
+      <c r="I45" s="12">
+        <f t="shared" si="4"/>
+        <v>0.74999999999999989</v>
+      </c>
+      <c r="J45" s="12"/>
     </row>
     <row r="46" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B46" s="16">
+      <c r="B46" s="12">
         <f t="shared" si="2"/>
         <v>20000</v>
       </c>
-      <c r="C46" s="16"/>
-      <c r="D46" s="17">
+      <c r="C46" s="12"/>
+      <c r="D46" s="11">
+        <f t="shared" si="5"/>
+        <v>9.999999999999998E-4</v>
+      </c>
+      <c r="E46" s="11"/>
+      <c r="G46" s="12">
         <f t="shared" si="3"/>
-        <v>9.999999999999998E-4</v>
-      </c>
-      <c r="E46" s="17"/>
+        <v>20</v>
+      </c>
+      <c r="H46" s="12"/>
+      <c r="I46" s="12">
+        <f t="shared" si="4"/>
+        <v>0.99999999999999978</v>
+      </c>
+      <c r="J46" s="12"/>
     </row>
     <row r="47" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B47" s="16">
+      <c r="B47" s="12">
         <f t="shared" si="2"/>
         <v>25000</v>
       </c>
-      <c r="C47" s="16"/>
-      <c r="D47" s="17">
+      <c r="C47" s="12"/>
+      <c r="D47" s="11">
+        <f t="shared" si="5"/>
+        <v>1.2499999999999998E-3</v>
+      </c>
+      <c r="E47" s="11"/>
+      <c r="G47" s="12">
         <f t="shared" si="3"/>
-        <v>1.2499999999999998E-3</v>
-      </c>
-      <c r="E47" s="17"/>
+        <v>25</v>
+      </c>
+      <c r="H47" s="12"/>
+      <c r="I47" s="12">
+        <f t="shared" si="4"/>
+        <v>1.2499999999999998</v>
+      </c>
+      <c r="J47" s="12"/>
     </row>
     <row r="48" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B48" s="16">
+      <c r="B48" s="12">
         <f t="shared" si="2"/>
         <v>30000</v>
       </c>
-      <c r="C48" s="16"/>
-      <c r="D48" s="17">
+      <c r="C48" s="12"/>
+      <c r="D48" s="11">
+        <f t="shared" si="5"/>
+        <v>1.4999999999999998E-3</v>
+      </c>
+      <c r="E48" s="11"/>
+      <c r="G48" s="12">
         <f t="shared" si="3"/>
-        <v>1.4999999999999998E-3</v>
-      </c>
-      <c r="E48" s="17"/>
-    </row>
-    <row r="49" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B49" s="16">
+        <v>30</v>
+      </c>
+      <c r="H48" s="12"/>
+      <c r="I48" s="12">
+        <f t="shared" si="4"/>
+        <v>1.4999999999999998</v>
+      </c>
+      <c r="J48" s="12"/>
+    </row>
+    <row r="49" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B49" s="12">
         <f t="shared" si="2"/>
         <v>35000</v>
       </c>
-      <c r="C49" s="16"/>
-      <c r="D49" s="17">
+      <c r="C49" s="12"/>
+      <c r="D49" s="11">
+        <f t="shared" si="5"/>
+        <v>1.7499999999999996E-3</v>
+      </c>
+      <c r="E49" s="11"/>
+      <c r="G49" s="12">
         <f t="shared" si="3"/>
-        <v>1.7499999999999996E-3</v>
-      </c>
-      <c r="E49" s="17"/>
-    </row>
-    <row r="50" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B50" s="16">
+        <v>35</v>
+      </c>
+      <c r="H49" s="12"/>
+      <c r="I49" s="12">
+        <f t="shared" si="4"/>
+        <v>1.7499999999999996</v>
+      </c>
+      <c r="J49" s="12"/>
+    </row>
+    <row r="50" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B50" s="12">
         <f t="shared" si="2"/>
         <v>40000</v>
       </c>
-      <c r="C50" s="16"/>
-      <c r="D50" s="17">
+      <c r="C50" s="12"/>
+      <c r="D50" s="11">
+        <f t="shared" si="5"/>
+        <v>1.9999999999999996E-3</v>
+      </c>
+      <c r="E50" s="11"/>
+      <c r="G50" s="12">
         <f t="shared" si="3"/>
-        <v>1.9999999999999996E-3</v>
-      </c>
-      <c r="E50" s="17"/>
-    </row>
-    <row r="52" spans="2:9" x14ac:dyDescent="0.3">
+        <v>40</v>
+      </c>
+      <c r="H50" s="12"/>
+      <c r="I50" s="12">
+        <f t="shared" si="4"/>
+        <v>1.9999999999999996</v>
+      </c>
+      <c r="J50" s="12"/>
+    </row>
+    <row r="52" spans="2:14" x14ac:dyDescent="0.3">
       <c r="I52" s="6"/>
     </row>
-    <row r="53" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B53" s="8" t="s">
+    <row r="53" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B53" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="C53" s="8"/>
-    </row>
-    <row r="54" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B54" s="8" t="s">
+      <c r="C53" s="15"/>
+      <c r="N53" s="6"/>
+    </row>
+    <row r="54" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B54" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="C54" s="8"/>
-    </row>
-    <row r="55" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B55" s="9">
+      <c r="C54" s="15"/>
+    </row>
+    <row r="55" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B55" s="19">
         <v>0</v>
       </c>
-      <c r="C55" s="9"/>
-    </row>
-    <row r="56" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B56" s="9">
-        <f t="shared" ref="B56:B63" si="4">(C21-D43)/D43</f>
+      <c r="C55" s="19"/>
+    </row>
+    <row r="56" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B56" s="19">
+        <f t="shared" ref="B56:B63" si="6">(C21-D43)/D43</f>
         <v>4.0000000000000327E-2</v>
       </c>
-      <c r="C56" s="9"/>
-    </row>
-    <row r="57" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B57" s="9">
-        <f t="shared" si="4"/>
+      <c r="C56" s="19"/>
+    </row>
+    <row r="57" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B57" s="19">
+        <f t="shared" si="6"/>
         <v>2.1684043449710094E-16</v>
       </c>
-      <c r="C57" s="9"/>
-    </row>
-    <row r="58" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B58" s="9">
-        <f t="shared" si="4"/>
+      <c r="C57" s="19"/>
+    </row>
+    <row r="58" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B58" s="19">
+        <f t="shared" si="6"/>
         <v>1.3333333333333515E-2</v>
       </c>
-      <c r="C58" s="9"/>
-    </row>
-    <row r="59" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B59" s="9">
-        <f t="shared" si="4"/>
+      <c r="C58" s="19"/>
+    </row>
+    <row r="59" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B59" s="19">
+        <f t="shared" si="6"/>
         <v>1.0000000000000245E-2</v>
       </c>
-      <c r="C59" s="9"/>
-    </row>
-    <row r="60" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B60" s="9">
-        <f t="shared" si="4"/>
+      <c r="C59" s="19"/>
+    </row>
+    <row r="60" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B60" s="19">
+        <f t="shared" si="6"/>
         <v>2.400000000000024E-2</v>
       </c>
-      <c r="C60" s="9"/>
-    </row>
-    <row r="61" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B61" s="9">
-        <f t="shared" si="4"/>
+      <c r="C60" s="19"/>
+    </row>
+    <row r="61" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B61" s="19">
+        <f t="shared" si="6"/>
         <v>2.6666666666666883E-2</v>
       </c>
-      <c r="C61" s="9"/>
-    </row>
-    <row r="62" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B62" s="9">
-        <f t="shared" si="4"/>
+      <c r="C61" s="19"/>
+    </row>
+    <row r="62" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B62" s="19">
+        <f t="shared" si="6"/>
         <v>1.142857142857171E-2</v>
       </c>
-      <c r="C62" s="9"/>
-    </row>
-    <row r="63" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B63" s="9">
-        <f t="shared" si="4"/>
+      <c r="C62" s="19"/>
+    </row>
+    <row r="63" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B63" s="19">
+        <f t="shared" si="6"/>
         <v>2.5000000000000071E-2</v>
       </c>
-      <c r="C63" s="9"/>
+      <c r="C63" s="19"/>
     </row>
     <row r="65" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B65" s="13" t="s">
+      <c r="B65" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="C65" s="13"/>
-      <c r="D65" s="13"/>
+      <c r="C65" s="10"/>
+      <c r="D65" s="10"/>
     </row>
     <row r="66" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B66" s="13" t="s">
+      <c r="B66" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="C66" s="13"/>
-      <c r="D66" s="13"/>
+      <c r="C66" s="10"/>
+      <c r="D66" s="10"/>
     </row>
     <row r="67" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B67" s="19" t="s">
+      <c r="B67" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="C67" s="19" t="s">
+      <c r="C67" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="D67" s="19" t="s">
+      <c r="D67" s="9" t="s">
         <v>30</v>
       </c>
     </row>
@@ -2534,7 +2651,7 @@
       <c r="C69" s="3">
         <v>5</v>
       </c>
-      <c r="D69" s="18">
+      <c r="D69" s="8">
         <f>B69/C69</f>
         <v>5.2000000000000005E-2</v>
       </c>
@@ -2546,8 +2663,8 @@
       <c r="C70" s="3">
         <v>10</v>
       </c>
-      <c r="D70" s="18">
-        <f t="shared" ref="D70:D76" si="5">B70/C70</f>
+      <c r="D70" s="8">
+        <f t="shared" ref="D70:D76" si="7">B70/C70</f>
         <v>0.05</v>
       </c>
     </row>
@@ -2558,8 +2675,8 @@
       <c r="C71" s="3">
         <v>15</v>
       </c>
-      <c r="D71" s="18">
-        <f t="shared" si="5"/>
+      <c r="D71" s="8">
+        <f t="shared" si="7"/>
         <v>5.0666666666666665E-2</v>
       </c>
     </row>
@@ -2570,8 +2687,8 @@
       <c r="C72" s="3">
         <v>20</v>
       </c>
-      <c r="D72" s="18">
-        <f t="shared" si="5"/>
+      <c r="D72" s="8">
+        <f t="shared" si="7"/>
         <v>5.0500000000000003E-2</v>
       </c>
     </row>
@@ -2582,8 +2699,8 @@
       <c r="C73" s="3">
         <v>25</v>
       </c>
-      <c r="D73" s="18">
-        <f t="shared" si="5"/>
+      <c r="D73" s="8">
+        <f t="shared" si="7"/>
         <v>5.1200000000000002E-2</v>
       </c>
     </row>
@@ -2594,8 +2711,8 @@
       <c r="C74" s="3">
         <v>30</v>
       </c>
-      <c r="D74" s="18">
-        <f t="shared" si="5"/>
+      <c r="D74" s="8">
+        <f t="shared" si="7"/>
         <v>5.1333333333333335E-2</v>
       </c>
     </row>
@@ -2606,8 +2723,8 @@
       <c r="C75" s="3">
         <v>35</v>
       </c>
-      <c r="D75" s="18">
-        <f t="shared" si="5"/>
+      <c r="D75" s="8">
+        <f t="shared" si="7"/>
         <v>5.0571428571428573E-2</v>
       </c>
     </row>
@@ -2618,24 +2735,48 @@
       <c r="C76" s="3">
         <v>40</v>
       </c>
-      <c r="D76" s="18">
-        <f t="shared" si="5"/>
+      <c r="D76" s="8">
+        <f t="shared" si="7"/>
         <v>5.1249999999999997E-2</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="44">
-    <mergeCell ref="B65:D65"/>
-    <mergeCell ref="B66:D66"/>
-    <mergeCell ref="D47:E47"/>
-    <mergeCell ref="D48:E48"/>
-    <mergeCell ref="D49:E49"/>
-    <mergeCell ref="D50:E50"/>
-    <mergeCell ref="D42:E42"/>
-    <mergeCell ref="D43:E43"/>
-    <mergeCell ref="D44:E44"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="D46:E46"/>
+  <mergeCells count="66">
+    <mergeCell ref="G50:H50"/>
+    <mergeCell ref="I50:J50"/>
+    <mergeCell ref="G47:H47"/>
+    <mergeCell ref="I47:J47"/>
+    <mergeCell ref="G48:H48"/>
+    <mergeCell ref="I48:J48"/>
+    <mergeCell ref="G49:H49"/>
+    <mergeCell ref="I49:J49"/>
+    <mergeCell ref="G44:H44"/>
+    <mergeCell ref="I44:J44"/>
+    <mergeCell ref="G45:H45"/>
+    <mergeCell ref="I45:J45"/>
+    <mergeCell ref="G46:H46"/>
+    <mergeCell ref="I46:J46"/>
+    <mergeCell ref="G41:H41"/>
+    <mergeCell ref="I41:J41"/>
+    <mergeCell ref="G42:H42"/>
+    <mergeCell ref="I42:J42"/>
+    <mergeCell ref="G43:H43"/>
+    <mergeCell ref="I43:J43"/>
+    <mergeCell ref="D41:E41"/>
+    <mergeCell ref="B54:C54"/>
+    <mergeCell ref="B55:C55"/>
+    <mergeCell ref="B56:C56"/>
+    <mergeCell ref="B57:C57"/>
+    <mergeCell ref="B46:C46"/>
+    <mergeCell ref="B47:C47"/>
+    <mergeCell ref="B48:C48"/>
+    <mergeCell ref="B49:C49"/>
+    <mergeCell ref="B50:C50"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="B43:C43"/>
+    <mergeCell ref="B44:C44"/>
+    <mergeCell ref="B45:C45"/>
     <mergeCell ref="B2:G2"/>
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="B40:E40"/>
@@ -2643,26 +2784,24 @@
     <mergeCell ref="B32:E32"/>
     <mergeCell ref="B31:E31"/>
     <mergeCell ref="B33:C33"/>
-    <mergeCell ref="B53:C53"/>
     <mergeCell ref="B18:C18"/>
     <mergeCell ref="B16:G16"/>
     <mergeCell ref="E18:G18"/>
     <mergeCell ref="E4:G4"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B42:C42"/>
-    <mergeCell ref="B43:C43"/>
-    <mergeCell ref="B44:C44"/>
-    <mergeCell ref="B45:C45"/>
-    <mergeCell ref="B46:C46"/>
-    <mergeCell ref="B47:C47"/>
-    <mergeCell ref="B48:C48"/>
-    <mergeCell ref="B49:C49"/>
-    <mergeCell ref="B50:C50"/>
-    <mergeCell ref="D41:E41"/>
-    <mergeCell ref="B54:C54"/>
-    <mergeCell ref="B55:C55"/>
-    <mergeCell ref="B56:C56"/>
-    <mergeCell ref="B57:C57"/>
+    <mergeCell ref="G39:J39"/>
+    <mergeCell ref="G40:J40"/>
+    <mergeCell ref="D42:E42"/>
+    <mergeCell ref="D43:E43"/>
+    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="B65:D65"/>
+    <mergeCell ref="B66:D66"/>
+    <mergeCell ref="D47:E47"/>
+    <mergeCell ref="D48:E48"/>
+    <mergeCell ref="D49:E49"/>
+    <mergeCell ref="D50:E50"/>
+    <mergeCell ref="B53:C53"/>
     <mergeCell ref="B63:C63"/>
     <mergeCell ref="B58:C58"/>
     <mergeCell ref="B59:C59"/>

</xml_diff>